<commit_message>
fix: regenerate timesheet template with proper biweekly structure; parser now accepts date strings
Old template was a 4-column placeholder. New template has the full
biweekly structure (title, consultant, date fields, day rows, hour
columns) matching what TimesheetParseService expects. Parser updated
with resolveDate() to accept both Excel date serials and formatted
date strings so users can enter dates naturally. Deploy hook now runs
timesheets:generate-template on each deploy so the file is always fresh.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/web/storage/app/templates/timesheet_template.xlsx
+++ b/web/storage/app/templates/timesheet_template.xlsx
@@ -15,18 +15,60 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="4">
-  <si>
-    <t>Consultant</t>
-  </si>
-  <si>
-    <t>Pay Period Start</t>
-  </si>
-  <si>
-    <t>Pay Period End</t>
-  </si>
-  <si>
-    <t>Total Hours</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="18">
+  <si>
+    <t>BI-WEEKLY TIMESHEET</t>
+  </si>
+  <si>
+    <t>Consultant:</t>
+  </si>
+  <si>
+    <t>Pay Period Start:</t>
+  </si>
+  <si>
+    <t>2026-03-24</t>
+  </si>
+  <si>
+    <t>Pay Period End:</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>DAY</t>
+  </si>
+  <si>
+    <t>DESCRIPTION</t>
+  </si>
+  <si>
+    <t>HOURS</t>
+  </si>
+  <si>
+    <t>Mon</t>
+  </si>
+  <si>
+    <t>Tue</t>
+  </si>
+  <si>
+    <t>Wed</t>
+  </si>
+  <si>
+    <t>Thu</t>
+  </si>
+  <si>
+    <t>Fri</t>
+  </si>
+  <si>
+    <t>Sat</t>
+  </si>
+  <si>
+    <t>Sun</t>
+  </si>
+  <si>
+    <t>TOTAL HOURS:</t>
   </si>
 </sst>
 </file>
@@ -34,7 +76,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -44,16 +86,40 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -61,12 +127,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -366,21 +451,177 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="true" style="0"/>
+    <col min="2" max="2" width="10" customWidth="true" style="0"/>
+    <col min="3" max="3" width="30" customWidth="true" style="0"/>
+    <col min="7" max="7" width="12" customWidth="true" style="0"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:7">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F6" s="3" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="B13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="B14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="B16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="B17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="B21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="B22" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="B23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="F25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G25" s="1">
+        <f>SUM(G10:G23)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Timesheets: edit hours after import (T016); biweekly template dates (T017)
Admin PATCH timesheets/{id}/hours recomputes OT from snapshots; audit log; invoice guard. BiweeklyPayPeriod anchor for GenerateTimesheetTemplate F6/F7 and daily DATE column. Tests: TimesheetHoursUpdateTest, BiweeklyPayPeriodTest. Regenerate template locally: php artisan timesheets:generate-template

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/web/storage/app/templates/timesheet_template.xlsx
+++ b/web/storage/app/templates/timesheet_template.xlsx
@@ -26,13 +26,13 @@
     <t>Pay Period Start:</t>
   </si>
   <si>
-    <t>2026-03-24</t>
+    <t>2026-03-23</t>
   </si>
   <si>
     <t>Pay Period End:</t>
   </si>
   <si>
-    <t>2026-04-06</t>
+    <t>2026-04-05</t>
   </si>
   <si>
     <t>DATE</t>
@@ -75,7 +75,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy&quot;/&quot;mm&quot;/&quot;dd;@"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <b val="0"/>
@@ -146,12 +148,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -504,6 +507,9 @@
       </c>
     </row>
     <row r="10" spans="1:7">
+      <c r="A10" s="5">
+        <v>46104.0</v>
+      </c>
       <c r="B10" t="s">
         <v>10</v>
       </c>
@@ -512,6 +518,9 @@
       </c>
     </row>
     <row r="11" spans="1:7">
+      <c r="A11" s="5">
+        <v>46105.0</v>
+      </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
@@ -520,6 +529,9 @@
       </c>
     </row>
     <row r="12" spans="1:7">
+      <c r="A12" s="5">
+        <v>46106.0</v>
+      </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
@@ -528,6 +540,9 @@
       </c>
     </row>
     <row r="13" spans="1:7">
+      <c r="A13" s="5">
+        <v>46107.0</v>
+      </c>
       <c r="B13" t="s">
         <v>13</v>
       </c>
@@ -536,6 +551,9 @@
       </c>
     </row>
     <row r="14" spans="1:7">
+      <c r="A14" s="5">
+        <v>46108.0</v>
+      </c>
       <c r="B14" t="s">
         <v>14</v>
       </c>
@@ -544,6 +562,9 @@
       </c>
     </row>
     <row r="15" spans="1:7">
+      <c r="A15" s="5">
+        <v>46109.0</v>
+      </c>
       <c r="B15" t="s">
         <v>15</v>
       </c>
@@ -552,6 +573,9 @@
       </c>
     </row>
     <row r="16" spans="1:7">
+      <c r="A16" s="5">
+        <v>46110.0</v>
+      </c>
       <c r="B16" t="s">
         <v>16</v>
       </c>
@@ -560,6 +584,9 @@
       </c>
     </row>
     <row r="17" spans="1:7">
+      <c r="A17" s="5">
+        <v>46111.0</v>
+      </c>
       <c r="B17" t="s">
         <v>10</v>
       </c>
@@ -568,6 +595,9 @@
       </c>
     </row>
     <row r="18" spans="1:7">
+      <c r="A18" s="5">
+        <v>46112.0</v>
+      </c>
       <c r="B18" t="s">
         <v>11</v>
       </c>
@@ -576,6 +606,9 @@
       </c>
     </row>
     <row r="19" spans="1:7">
+      <c r="A19" s="5">
+        <v>46113.0</v>
+      </c>
       <c r="B19" t="s">
         <v>12</v>
       </c>
@@ -584,6 +617,9 @@
       </c>
     </row>
     <row r="20" spans="1:7">
+      <c r="A20" s="5">
+        <v>46114.0</v>
+      </c>
       <c r="B20" t="s">
         <v>13</v>
       </c>
@@ -592,6 +628,9 @@
       </c>
     </row>
     <row r="21" spans="1:7">
+      <c r="A21" s="5">
+        <v>46115.0</v>
+      </c>
       <c r="B21" t="s">
         <v>14</v>
       </c>
@@ -600,6 +639,9 @@
       </c>
     </row>
     <row r="22" spans="1:7">
+      <c r="A22" s="5">
+        <v>46116.0</v>
+      </c>
       <c r="B22" t="s">
         <v>15</v>
       </c>
@@ -608,6 +650,9 @@
       </c>
     </row>
     <row r="23" spans="1:7">
+      <c r="A23" s="5">
+        <v>46117.0</v>
+      </c>
       <c r="B23" t="s">
         <v>16</v>
       </c>

</xml_diff>